<commit_message>
docs(vaers): pre-send fixes — xlsx nonseverable/52.227-17 (was contradicting PDF), CPARS+reps block added to Vol II per Q69/Q203, Vol I re-rendered w/ PRA row; body 15/15 pages, fonts clean
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PuKJAXTWtKewKXACtap8EQ
</commit_message>
<xml_diff>
--- a/docs/responses/2026-09-04-cdc-vaers/out/Vol-II-Price-Quote-FrasierDigital.xlsx
+++ b/docs/responses/2026-09-04-cdc-vaers/out/Vol-II-Price-Quote-FrasierDigital.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Design, development, deployment, and compliance delivery of the Modernized VAERS Reporting Application per the PWS (severable services)</t>
+          <t>Design, development, deployment, and compliance delivery of the Modernized VAERS Reporting Application per the PWS (nonseverable services per Amendment 0001)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>None required — all custom code delivered open source per M-16-21; development on contractor equipment; laptops and PIV cards are Government-furnished</t>
+          <t>None required — all custom code delivered with Government rights per FAR 52.227-17 (Amendment 0001 Q&amp;A 91); development on contractor equipment; laptops and PIV cards are Government-furnished</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">

</xml_diff>